<commit_message>
Amikacin HDEI: follow UpToDate below CrCl 40, same as gentamicin
- CrCl 20-<40: 15-20 mg/kg q48h; CrCl <20: usual dose once, then individualise
- Removes the builder-added "<30 HDEI not recommended" row
- Reference table: HDEI row no longer shares the conventional 10-29 / <10 cells
- Same change in rules workbook and app; test checks amikacin vs gentamicin HDEI
- sw.js CACHE renal-v2 so installed phones update

Fixes #2

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/App/IV-ATB-Renal-App_RULES.xlsx
+++ b/App/IV-ATB-Renal-App_RULES.xlsx
@@ -1408,7 +1408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N105"/>
+  <dimension ref="A1:N107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1994,25 +1994,29 @@
         <v>5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>30</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>ไม่แนะนำสูตร HDEI เมื่อ CrCl &lt;30 — ใช้สูตร Conventional</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
+          <t>15-20 mg/kg q 48 h</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>q 48 h</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>(เพิ่มโดยผู้จัดทำ: ตารางเดิมเว้นว่าง) ตรวจสอบ</t>
-        </is>
-      </c>
+      <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
           <t>ตรวจสอบ</t>
@@ -2022,27 +2026,39 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>amoxiclav</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n"/>
+          <t>amikacin</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>HDEI (วันละครั้ง)</t>
+        </is>
+      </c>
       <c r="C14" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl ≥30): IV 1.2 g q 8 h</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
+          <t>ให้ครั้งเดียว แล้วปรับตามผู้ป่วย</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>ครั้งเดียว</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="inlineStr">
@@ -2054,27 +2070,39 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>amoxiclav</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n"/>
+          <t>amikacin</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>HDEI (วันละครั้ง)</t>
+        </is>
+      </c>
       <c r="C15" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E15" s="2" t="n">
-        <v>30</v>
-      </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>เริ่ม 1 g จากนั้น 500 mg q 12 h</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+          <t>ให้ครั้งเดียว แล้วปรับตามผู้ป่วย</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>ครั้งเดียว</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="inlineStr">
@@ -2091,17 +2119,17 @@
       </c>
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>10</v>
+        <v>9999</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>เริ่ม 1 g จากนั้น 500 mg q 12-24 h</t>
+          <t>ไม่ต้องปรับขนาด (CrCl ≥30): IV 1.2 g q 8 h</t>
         </is>
       </c>
       <c r="G16" s="2" t="n"/>
@@ -2118,26 +2146,22 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ampicillin</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>1-2 g q6h</t>
-        </is>
-      </c>
+          <t>amoxiclav</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
       <c r="C17" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>9999</v>
+        <v>30</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl ≥50): 1-2 g q 6 h</t>
+          <t>เริ่ม 1 g จากนั้น 500 mg q 12 h</t>
         </is>
       </c>
       <c r="G17" s="2" t="n"/>
@@ -2154,26 +2178,22 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ampicillin</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>1-2 g q6h</t>
-        </is>
-      </c>
+          <t>amoxiclav</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>1-2 g q 8 h</t>
+          <t>เริ่ม 1 g จากนั้น 500 mg q 12-24 h</t>
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
@@ -2199,17 +2219,17 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>30</v>
+        <v>9999</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>1-2 g q 12 h</t>
+          <t>ไม่ต้องปรับขนาด (CrCl ≥50): 1-2 g q 6 h</t>
         </is>
       </c>
       <c r="G19" s="2" t="n"/>
@@ -2235,17 +2255,17 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>1-2 g q 24 h</t>
+          <t>1-2 g q 8 h</t>
         </is>
       </c>
       <c r="G20" s="2" t="n"/>
@@ -2267,21 +2287,21 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>2 g q4h (รุนแรง)</t>
+          <t>1-2 g q6h</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>9999</v>
+        <v>30</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl ≥50): 2 g q 4 h</t>
+          <t>1-2 g q 12 h</t>
         </is>
       </c>
       <c r="G21" s="2" t="n"/>
@@ -2303,21 +2323,21 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2 g q4h (รุนแรง)</t>
+          <t>1-2 g q6h</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2 g q 6 h</t>
+          <t>1-2 g q 24 h</t>
         </is>
       </c>
       <c r="G22" s="2" t="n"/>
@@ -2343,17 +2363,17 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>30</v>
+        <v>9999</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2 g q 8 h</t>
+          <t>ไม่ต้องปรับขนาด (CrCl ≥50): 2 g q 4 h</t>
         </is>
       </c>
       <c r="G23" s="2" t="n"/>
@@ -2379,17 +2399,17 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2 g q 12 h</t>
+          <t>2 g q 6 h</t>
         </is>
       </c>
       <c r="G24" s="2" t="n"/>
@@ -2406,22 +2426,26 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>cefazolin</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n"/>
+          <t>ampicillin</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2 g q4h (รุนแรง)</t>
+        </is>
+      </c>
       <c r="C25" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>9999</v>
+        <v>30</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl ≥50): 1-2 g q 8 h</t>
+          <t>2 g q 8 h</t>
         </is>
       </c>
       <c r="G25" s="2" t="n"/>
@@ -2438,22 +2462,26 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>cefazolin</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n"/>
+          <t>ampicillin</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>2 g q4h (รุนแรง)</t>
+        </is>
+      </c>
       <c r="C26" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>1-2 g q 8-12 h</t>
+          <t>2 g q 12 h</t>
         </is>
       </c>
       <c r="G26" s="2" t="n"/>
@@ -2475,17 +2503,17 @@
       </c>
       <c r="B27" s="2" t="n"/>
       <c r="C27" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>30</v>
+        <v>9999</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>500 mg-1 g q 12 h (2 g q 12 h ถ้ารุนแรง)</t>
+          <t>ไม่ต้องปรับขนาด (CrCl ≥50): 1-2 g q 8 h</t>
         </is>
       </c>
       <c r="G27" s="2" t="n"/>
@@ -2507,17 +2535,17 @@
       </c>
       <c r="B28" s="2" t="n"/>
       <c r="C28" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>500 mg-1 g q 24 h</t>
+          <t>1-2 g q 8-12 h</t>
         </is>
       </c>
       <c r="G28" s="2" t="n"/>
@@ -2534,26 +2562,22 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>cefotaxime</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>1-2 g q8h</t>
-        </is>
-      </c>
+          <t>cefazolin</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n"/>
       <c r="C29" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>9999</v>
+        <v>30</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 1-2 g q 8 h</t>
+          <t>500 mg-1 g q 12 h (2 g q 12 h ถ้ารุนแรง)</t>
         </is>
       </c>
       <c r="G29" s="2" t="n"/>
@@ -2570,26 +2594,22 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>cefotaxime</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>1-2 g q8h</t>
-        </is>
-      </c>
+          <t>cefazolin</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n"/>
       <c r="C30" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E30" s="2" t="n">
-        <v>50</v>
-      </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>1-2 g q 12 h</t>
+          <t>500 mg-1 g q 24 h</t>
         </is>
       </c>
       <c r="G30" s="2" t="n"/>
@@ -2615,17 +2635,17 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>10</v>
+        <v>9999</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>1-2 g q 24 h</t>
+          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 1-2 g q 8 h</t>
         </is>
       </c>
       <c r="G31" s="2" t="n"/>
@@ -2647,21 +2667,21 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>1-2 g q6h</t>
+          <t>1-2 g q8h</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E32" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="E32" s="2" t="n">
-        <v>9999</v>
-      </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 1-2 g q 6 h</t>
+          <t>1-2 g q 12 h</t>
         </is>
       </c>
       <c r="G32" s="2" t="n"/>
@@ -2683,21 +2703,21 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>1-2 g q6h</t>
+          <t>1-2 g q8h</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E33" s="2" t="n">
-        <v>50</v>
-      </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>1-2 g q 8 h</t>
+          <t>1-2 g q 24 h</t>
         </is>
       </c>
       <c r="G33" s="2" t="n"/>
@@ -2723,17 +2743,17 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>10</v>
+        <v>9999</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>1-2 g q 12 h</t>
+          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 1-2 g q 6 h</t>
         </is>
       </c>
       <c r="G34" s="2" t="n"/>
@@ -2755,21 +2775,21 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>2 g q4h (รุนแรง)</t>
+          <t>1-2 g q6h</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E35" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="E35" s="2" t="n">
-        <v>9999</v>
-      </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 2 g q 4 h</t>
+          <t>1-2 g q 8 h</t>
         </is>
       </c>
       <c r="G35" s="2" t="n"/>
@@ -2791,21 +2811,21 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2 g q4h (รุนแรง)</t>
+          <t>1-2 g q6h</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E36" s="2" t="n">
-        <v>50</v>
-      </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2 g q 6-8 h</t>
+          <t>1-2 g q 12 h</t>
         </is>
       </c>
       <c r="G36" s="2" t="n"/>
@@ -2831,17 +2851,17 @@
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>10</v>
+        <v>9999</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2 g q 12 h</t>
+          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 2 g q 4 h</t>
         </is>
       </c>
       <c r="G37" s="2" t="n"/>
@@ -2858,26 +2878,26 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ceftazidime</t>
+          <t>cefotaxime</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>1 g q8h</t>
+          <t>2 g q4h (รุนแรง)</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>9999</v>
+        <v>50</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 1 g q 8 h</t>
+          <t>2 g q 6-8 h</t>
         </is>
       </c>
       <c r="G38" s="2" t="n"/>
@@ -2894,26 +2914,26 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ceftazidime</t>
+          <t>cefotaxime</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>1 g q8h</t>
+          <t>2 g q4h (รุนแรง)</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>1 g q 12 h (CrCl 31-50)</t>
+          <t>2 g q 12 h</t>
         </is>
       </c>
       <c r="G39" s="2" t="n"/>
@@ -2939,17 +2959,17 @@
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>31</v>
+        <v>9999</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>1 g q 24 h (CrCl 16-30)</t>
+          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 1 g q 8 h</t>
         </is>
       </c>
       <c r="G40" s="2" t="n"/>
@@ -2975,17 +2995,17 @@
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>500 mg q 24 h (CrCl ≤15)</t>
+          <t>1 g q 12 h (CrCl 31-50)</t>
         </is>
       </c>
       <c r="G41" s="2" t="n"/>
@@ -3007,21 +3027,21 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2 g q8h (Pseudomonas/รุนแรง)</t>
+          <t>1 g q8h</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>9999</v>
+        <v>31</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 2 g q 8 h</t>
+          <t>1 g q 24 h (CrCl 16-30)</t>
         </is>
       </c>
       <c r="G42" s="2" t="n"/>
@@ -3043,21 +3063,21 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2 g q8h (Pseudomonas/รุนแรง)</t>
+          <t>1 g q8h</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2 g q 12 h (CrCl 31-50)</t>
+          <t>500 mg q 24 h (CrCl ≤15)</t>
         </is>
       </c>
       <c r="G43" s="2" t="n"/>
@@ -3083,17 +3103,17 @@
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>31</v>
+        <v>9999</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2 g q 24 h (CrCl 16-30)</t>
+          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 2 g q 8 h</t>
         </is>
       </c>
       <c r="G44" s="2" t="n"/>
@@ -3119,17 +3139,17 @@
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>1 g q 24 h (CrCl ≤15)</t>
+          <t>2 g q 12 h (CrCl 31-50)</t>
         </is>
       </c>
       <c r="G45" s="2" t="n"/>
@@ -3146,22 +3166,26 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>ciprofloxacin</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="n"/>
+          <t>ceftazidime</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>2 g q8h (Pseudomonas/รุนแรง)</t>
+        </is>
+      </c>
       <c r="C46" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>9999</v>
+        <v>31</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>400 mg q 8-12 h (CrCl ≥30)</t>
+          <t>2 g q 24 h (CrCl 16-30)</t>
         </is>
       </c>
       <c r="G46" s="2" t="n"/>
@@ -3178,22 +3202,26 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>ciprofloxacin</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="n"/>
+          <t>ceftazidime</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>2 g q8h (Pseudomonas/รุนแรง)</t>
+        </is>
+      </c>
       <c r="C47" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>200-400 mg q 12-24 h</t>
+          <t>1 g q 24 h (CrCl ≤15)</t>
         </is>
       </c>
       <c r="G47" s="2" t="n"/>
@@ -3210,36 +3238,28 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>colistin</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>ขนาดคงระดับ (แบ่ง 2 ครั้ง/วัน)</t>
-        </is>
-      </c>
+          <t>ciprofloxacin</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>9999</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>360 mg CBA/วัน (2.4 vial)</t>
+          <t>400 mg q 8-12 h (CrCl ≥30)</t>
         </is>
       </c>
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="2" t="n"/>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>ขนาดนำ 300 mg CBA = 2 vial (เริ่มขนาดคงระดับ 12 ชม. หลังขนาดนำ)</t>
-        </is>
-      </c>
+      <c r="J48" s="2" t="n"/>
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
@@ -3250,36 +3270,28 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>colistin</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>ขนาดคงระดับ (แบ่ง 2 ครั้ง/วัน)</t>
-        </is>
-      </c>
+          <t>ciprofloxacin</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>340 mg CBA/วัน (2.25 vial)</t>
+          <t>200-400 mg q 12-24 h</t>
         </is>
       </c>
       <c r="G49" s="2" t="n"/>
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="2" t="n"/>
-      <c r="J49" s="2" t="inlineStr">
-        <is>
-          <t>ขนาดนำ 300 mg CBA = 2 vial (เริ่ม 12 ชม. หลังขนาดนำ)</t>
-        </is>
-      </c>
+      <c r="J49" s="2" t="n"/>
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
@@ -3299,17 +3311,17 @@
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>80</v>
+        <v>9999</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>300 mg CBA/วัน (2 vial)</t>
+          <t>360 mg CBA/วัน (2.4 vial)</t>
         </is>
       </c>
       <c r="G50" s="2" t="n"/>
@@ -3317,7 +3329,7 @@
       <c r="I50" s="2" t="n"/>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>ขนาดนำ 300 mg CBA = 2 vial</t>
+          <t>ขนาดนำ 300 mg CBA = 2 vial (เริ่มขนาดคงระดับ 12 ชม. หลังขนาดนำ)</t>
         </is>
       </c>
       <c r="K50" s="2" t="n"/>
@@ -3339,17 +3351,17 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>275 mg CBA/วัน (1.8 vial)</t>
+          <t>340 mg CBA/วัน (2.25 vial)</t>
         </is>
       </c>
       <c r="G51" s="2" t="n"/>
@@ -3357,7 +3369,7 @@
       <c r="I51" s="2" t="n"/>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>ขนาดนำ 300 mg CBA = 2 vial</t>
+          <t>ขนาดนำ 300 mg CBA = 2 vial (เริ่ม 12 ชม. หลังขนาดนำ)</t>
         </is>
       </c>
       <c r="K51" s="2" t="n"/>
@@ -3379,17 +3391,17 @@
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>245 mg CBA/วัน (1.6 vial)</t>
+          <t>300 mg CBA/วัน (2 vial)</t>
         </is>
       </c>
       <c r="G52" s="2" t="n"/>
@@ -3419,17 +3431,17 @@
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>220 mg CBA/วัน (1.5 vial)</t>
+          <t>275 mg CBA/วัน (1.8 vial)</t>
         </is>
       </c>
       <c r="G53" s="2" t="n"/>
@@ -3459,17 +3471,17 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>195 mg CBA/วัน (1.3 vial)</t>
+          <t>245 mg CBA/วัน (1.6 vial)</t>
         </is>
       </c>
       <c r="G54" s="2" t="n"/>
@@ -3499,17 +3511,17 @@
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>175 mg CBA/วัน (1.2 vial)</t>
+          <t>220 mg CBA/วัน (1.5 vial)</t>
         </is>
       </c>
       <c r="G55" s="2" t="n"/>
@@ -3539,17 +3551,17 @@
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>160 mg CBA/วัน (1.1 vial)</t>
+          <t>195 mg CBA/วัน (1.3 vial)</t>
         </is>
       </c>
       <c r="G56" s="2" t="n"/>
@@ -3579,17 +3591,17 @@
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>145 mg CBA/วัน (1 vial)</t>
+          <t>175 mg CBA/วัน (1.2 vial)</t>
         </is>
       </c>
       <c r="G57" s="2" t="n"/>
@@ -3619,17 +3631,17 @@
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>130 mg CBA/วัน (0.9 vial)</t>
+          <t>160 mg CBA/วัน (1.1 vial)</t>
         </is>
       </c>
       <c r="G58" s="2" t="n"/>
@@ -3650,28 +3662,36 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>ertapenem</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="n"/>
+          <t>colistin</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>ขนาดคงระดับ (แบ่ง 2 ครั้ง/วัน)</t>
+        </is>
+      </c>
       <c r="C59" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>9999</v>
+        <v>10</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>1 g วันละครั้ง (CrCl &gt;30, ไม่เปลี่ยน)</t>
+          <t>145 mg CBA/วัน (1 vial)</t>
         </is>
       </c>
       <c r="G59" s="2" t="n"/>
       <c r="H59" s="2" t="n"/>
       <c r="I59" s="2" t="n"/>
-      <c r="J59" s="2" t="n"/>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>ขนาดนำ 300 mg CBA = 2 vial</t>
+        </is>
+      </c>
       <c r="K59" s="2" t="n"/>
       <c r="L59" s="2" t="inlineStr">
         <is>
@@ -3682,28 +3702,36 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>ertapenem</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="n"/>
+          <t>colistin</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>ขนาดคงระดับ (แบ่ง 2 ครั้ง/วัน)</t>
+        </is>
+      </c>
       <c r="C60" s="2" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D60" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>500 mg วันละครั้ง (CrCl ≤30)</t>
+          <t>130 mg CBA/วัน (0.9 vial)</t>
         </is>
       </c>
       <c r="G60" s="2" t="n"/>
       <c r="H60" s="2" t="n"/>
       <c r="I60" s="2" t="n"/>
-      <c r="J60" s="2" t="n"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>ขนาดนำ 300 mg CBA = 2 vial</t>
+        </is>
+      </c>
       <c r="K60" s="2" t="n"/>
       <c r="L60" s="2" t="inlineStr">
         <is>
@@ -3714,26 +3742,22 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>gentamicin</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>Conventional (3-5 mg/kg/วัน แบ่ง q8h)</t>
-        </is>
-      </c>
+          <t>ertapenem</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n"/>
       <c r="C61" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>9999</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl ≥60): ขนาดปกติ q 8 h</t>
+          <t>1 g วันละครั้ง (CrCl &gt;30, ไม่เปลี่ยน)</t>
         </is>
       </c>
       <c r="G61" s="2" t="n"/>
@@ -3750,26 +3774,22 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>gentamicin</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Conventional (3-5 mg/kg/วัน แบ่ง q8h)</t>
-        </is>
-      </c>
+          <t>ertapenem</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>ขนาดปกติ q 12 h</t>
+          <t>500 mg วันละครั้ง (CrCl ≤30)</t>
         </is>
       </c>
       <c r="G62" s="2" t="n"/>
@@ -3795,17 +3815,17 @@
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>50</v>
+        <v>9999</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>ขนาดปกติ q 12 h</t>
+          <t>ไม่ต้องปรับขนาด (CrCl ≥60): ขนาดปกติ q 8 h</t>
         </is>
       </c>
       <c r="G63" s="2" t="n"/>
@@ -3831,17 +3851,17 @@
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>ขนาดปกติ q 24 h</t>
+          <t>ขนาดปกติ q 12 h</t>
         </is>
       </c>
       <c r="G64" s="2" t="n"/>
@@ -3867,17 +3887,17 @@
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>ขนาดปกติ q 24 h</t>
+          <t>ขนาดปกติ q 12 h</t>
         </is>
       </c>
       <c r="G65" s="2" t="n"/>
@@ -3903,17 +3923,17 @@
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>ขนาดปกติ q 36-48 h</t>
+          <t>ขนาดปกติ q 24 h</t>
         </is>
       </c>
       <c r="G66" s="2" t="n"/>
@@ -3939,17 +3959,17 @@
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>ขนาดปกติ q 36-48 h</t>
+          <t>ขนาดปกติ q 24 h</t>
         </is>
       </c>
       <c r="G67" s="2" t="n"/>
@@ -3971,34 +3991,26 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>HDEI (5-7 mg/kg q24h)</t>
+          <t>Conventional (3-5 mg/kg/วัน แบ่ง q8h)</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>5-7 mg/kg q 24 h (CrCl ≥60)</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>q 24 h</t>
-        </is>
-      </c>
+          <t>ขนาดปกติ q 36-48 h</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="n"/>
+      <c r="H68" s="2" t="n"/>
+      <c r="I68" s="2" t="n"/>
       <c r="J68" s="2" t="n"/>
       <c r="K68" s="2" t="n"/>
       <c r="L68" s="2" t="inlineStr">
@@ -4015,34 +4027,26 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>HDEI (5-7 mg/kg q24h)</t>
+          <t>Conventional (3-5 mg/kg/วัน แบ่ง q8h)</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>5-7 mg/kg q 36 h</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H69" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>q 36 h</t>
-        </is>
-      </c>
+          <t>ขนาดปกติ q 36-48 h</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="n"/>
+      <c r="I69" s="2" t="n"/>
       <c r="J69" s="2" t="n"/>
       <c r="K69" s="2" t="n"/>
       <c r="L69" s="2" t="inlineStr">
@@ -4063,17 +4067,17 @@
         </is>
       </c>
       <c r="C70" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>50</v>
+        <v>9999</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>5-7 mg/kg q 36 h</t>
+          <t>5-7 mg/kg q 24 h (CrCl ≥60)</t>
         </is>
       </c>
       <c r="G70" s="2" t="n">
@@ -4084,7 +4088,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>q 36 h</t>
+          <t>q 24 h</t>
         </is>
       </c>
       <c r="J70" s="2" t="n"/>
@@ -4107,17 +4111,17 @@
         </is>
       </c>
       <c r="C71" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>5-7 mg/kg q 48 h</t>
+          <t>5-7 mg/kg q 36 h</t>
         </is>
       </c>
       <c r="G71" s="2" t="n">
@@ -4128,7 +4132,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>q 48 h</t>
+          <t>q 36 h</t>
         </is>
       </c>
       <c r="J71" s="2" t="n"/>
@@ -4151,17 +4155,17 @@
         </is>
       </c>
       <c r="C72" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>5-7 mg/kg q 48 h</t>
+          <t>5-7 mg/kg q 36 h</t>
         </is>
       </c>
       <c r="G72" s="2" t="n">
@@ -4172,7 +4176,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>q 48 h</t>
+          <t>q 36 h</t>
         </is>
       </c>
       <c r="J72" s="2" t="n"/>
@@ -4195,17 +4199,17 @@
         </is>
       </c>
       <c r="C73" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>ให้ครั้งเดียว แล้วปรับตามผู้ป่วย</t>
+          <t>5-7 mg/kg q 48 h</t>
         </is>
       </c>
       <c r="G73" s="2" t="n">
@@ -4216,7 +4220,7 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>ครั้งเดียว</t>
+          <t>q 48 h</t>
         </is>
       </c>
       <c r="J73" s="2" t="n"/>
@@ -4239,17 +4243,17 @@
         </is>
       </c>
       <c r="C74" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D74" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>ให้ครั้งเดียว แล้วปรับตามผู้ป่วย</t>
+          <t>5-7 mg/kg q 48 h</t>
         </is>
       </c>
       <c r="G74" s="2" t="n">
@@ -4260,7 +4264,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>ครั้งเดียว</t>
+          <t>q 48 h</t>
         </is>
       </c>
       <c r="J74" s="2" t="n"/>
@@ -4274,31 +4278,39 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>meropenem</t>
+          <t>gentamicin</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>1 g q8h</t>
+          <t>HDEI (5-7 mg/kg q24h)</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D75" s="2" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 1 g q 8 h</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="n"/>
-      <c r="H75" s="2" t="n"/>
-      <c r="I75" s="2" t="n"/>
+          <t>ให้ครั้งเดียว แล้วปรับตามผู้ป่วย</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>ครั้งเดียว</t>
+        </is>
+      </c>
       <c r="J75" s="2" t="n"/>
       <c r="K75" s="2" t="n"/>
       <c r="L75" s="2" t="inlineStr">
@@ -4310,31 +4322,39 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>meropenem</t>
+          <t>gentamicin</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>1 g q8h</t>
+          <t>HDEI (5-7 mg/kg q24h)</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D76" s="2" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>1 g q 12 h (CrCl 26-50)</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="n"/>
-      <c r="H76" s="2" t="n"/>
-      <c r="I76" s="2" t="n"/>
+          <t>ให้ครั้งเดียว แล้วปรับตามผู้ป่วย</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>ครั้งเดียว</t>
+        </is>
+      </c>
       <c r="J76" s="2" t="n"/>
       <c r="K76" s="2" t="n"/>
       <c r="L76" s="2" t="inlineStr">
@@ -4355,17 +4375,17 @@
         </is>
       </c>
       <c r="C77" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D77" s="2" t="n">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>26</v>
+        <v>9999</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>500 mg q 12 h (CrCl 10-25)</t>
+          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 1 g q 8 h</t>
         </is>
       </c>
       <c r="G77" s="2" t="n"/>
@@ -4391,17 +4411,17 @@
         </is>
       </c>
       <c r="C78" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D78" s="2" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>500 mg q 24 h</t>
+          <t>1 g q 12 h (CrCl 26-50)</t>
         </is>
       </c>
       <c r="G78" s="2" t="n"/>
@@ -4423,21 +4443,21 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>2 g q8h</t>
+          <t>1 g q8h</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D79" s="2" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>9999</v>
+        <v>26</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 2 g q 8 h</t>
+          <t>500 mg q 12 h (CrCl 10-25)</t>
         </is>
       </c>
       <c r="G79" s="2" t="n"/>
@@ -4459,21 +4479,21 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>2 g q8h</t>
+          <t>1 g q8h</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D80" s="2" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2 g q 12 h (CrCl 26-50)</t>
+          <t>500 mg q 24 h</t>
         </is>
       </c>
       <c r="G80" s="2" t="n"/>
@@ -4499,17 +4519,17 @@
         </is>
       </c>
       <c r="C81" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D81" s="2" t="n">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>26</v>
+        <v>9999</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>1 g q 12 h (CrCl 10-25)</t>
+          <t>ไม่ต้องปรับขนาด (CrCl &gt;50): 2 g q 8 h</t>
         </is>
       </c>
       <c r="G81" s="2" t="n"/>
@@ -4535,17 +4555,17 @@
         </is>
       </c>
       <c r="C82" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D82" s="2" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>1 g q 24 h หรือ 500 mg q 12 h</t>
+          <t>2 g q 12 h (CrCl 26-50)</t>
         </is>
       </c>
       <c r="G82" s="2" t="n"/>
@@ -4562,22 +4582,26 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>penicillinG</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="n"/>
+          <t>meropenem</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>2 g q8h</t>
+        </is>
+      </c>
       <c r="C83" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D83" s="2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>9999</v>
+        <v>26</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl &gt;50)</t>
+          <t>1 g q 12 h (CrCl 10-25)</t>
         </is>
       </c>
       <c r="G83" s="2" t="n"/>
@@ -4594,22 +4618,26 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>penicillinG</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="n"/>
+          <t>meropenem</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>2 g q8h</t>
+        </is>
+      </c>
       <c r="C84" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D84" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>50-75% ของขนาดปกติ</t>
+          <t>1 g q 24 h หรือ 500 mg q 12 h</t>
         </is>
       </c>
       <c r="G84" s="2" t="n"/>
@@ -4631,17 +4659,17 @@
       </c>
       <c r="B85" s="2" t="n"/>
       <c r="C85" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D85" s="2" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>30</v>
+        <v>9999</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>25-50% ของขนาดปกติ</t>
+          <t>ไม่ต้องปรับขนาด (CrCl &gt;50)</t>
         </is>
       </c>
       <c r="G85" s="2" t="n"/>
@@ -4663,17 +4691,17 @@
       </c>
       <c r="B86" s="2" t="n"/>
       <c r="C86" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D86" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>20-25% ของขนาดปกติ</t>
+          <t>50-75% ของขนาดปกติ</t>
         </is>
       </c>
       <c r="G86" s="2" t="n"/>
@@ -4690,26 +4718,22 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>piptazo</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>3.375 g q6h</t>
-        </is>
-      </c>
+          <t>penicillinG</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="n"/>
       <c r="C87" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D87" s="2" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>9999</v>
+        <v>30</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl ≥40): 3.375 g q 6 h</t>
+          <t>25-50% ของขนาดปกติ</t>
         </is>
       </c>
       <c r="G87" s="2" t="n"/>
@@ -4726,26 +4750,22 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>piptazo</t>
-        </is>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>3.375 g q6h</t>
-        </is>
-      </c>
+          <t>penicillinG</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n"/>
       <c r="C88" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D88" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2.25 g q 6 h</t>
+          <t>20-25% ของขนาดปกติ</t>
         </is>
       </c>
       <c r="G88" s="2" t="n"/>
@@ -4771,17 +4791,17 @@
         </is>
       </c>
       <c r="C89" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D89" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>30</v>
+        <v>9999</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2.25 g q 6 h</t>
+          <t>ไม่ต้องปรับขนาด (CrCl ≥40): 3.375 g q 6 h</t>
         </is>
       </c>
       <c r="G89" s="2" t="n"/>
@@ -4807,17 +4827,17 @@
         </is>
       </c>
       <c r="C90" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D90" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2.25 g q 8 h</t>
+          <t>2.25 g q 6 h</t>
         </is>
       </c>
       <c r="G90" s="2" t="n"/>
@@ -4839,21 +4859,21 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>4.5 g q6h</t>
+          <t>3.375 g q6h</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D91" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>9999</v>
+        <v>30</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด (CrCl ≥40): 4.5 g q 6 h</t>
+          <t>2.25 g q 6 h</t>
         </is>
       </c>
       <c r="G91" s="2" t="n"/>
@@ -4875,21 +4895,21 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>4.5 g q6h</t>
+          <t>3.375 g q6h</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D92" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>4.5 g q 8 h หรือ 3.375 g q 6 h</t>
+          <t>2.25 g q 8 h</t>
         </is>
       </c>
       <c r="G92" s="2" t="n"/>
@@ -4915,17 +4935,17 @@
         </is>
       </c>
       <c r="C93" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D93" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>30</v>
+        <v>9999</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>4.5 g q 8 h หรือ 3.375 g q 6 h</t>
+          <t>ไม่ต้องปรับขนาด (CrCl ≥40): 4.5 g q 6 h</t>
         </is>
       </c>
       <c r="G93" s="2" t="n"/>
@@ -4951,17 +4971,17 @@
         </is>
       </c>
       <c r="C94" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D94" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>4.5 g q 12 h หรือ 2.25 g q 6 h</t>
+          <t>4.5 g q 8 h หรือ 3.375 g q 6 h</t>
         </is>
       </c>
       <c r="G94" s="2" t="n"/>
@@ -4978,100 +4998,74 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>vancomycin</t>
-        </is>
-      </c>
-      <c r="B95" s="2" t="n"/>
+          <t>piptazo</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>4.5 g q6h</t>
+        </is>
+      </c>
       <c r="C95" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D95" s="2" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>9999</v>
+        <v>30</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>15-20 mg/kg q 8-12 h</t>
-        </is>
-      </c>
-      <c r="G95" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="H95" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="I95" s="2" t="inlineStr">
-        <is>
-          <t>q 8-12 h</t>
-        </is>
-      </c>
-      <c r="J95" s="2" t="inlineStr">
-        <is>
-          <t>25-30 mg/kg ครั้งเดียว — เฉพาะผู้ป่วยวิกฤตที่สงสัย/ยืนยันติดเชื้อ MRSA รุนแรง; คิดตามน้ำหนักจริง; สูงสุด 3 g; เริ่มขนาดคงระดับในรอบถัดไป</t>
-        </is>
-      </c>
+          <t>4.5 g q 8 h หรือ 3.375 g q 6 h</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="n"/>
+      <c r="H95" s="2" t="n"/>
+      <c r="I95" s="2" t="n"/>
+      <c r="J95" s="2" t="n"/>
       <c r="K95" s="2" t="n"/>
       <c r="L95" s="2" t="inlineStr">
         <is>
           <t>ตรวจสอบ</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>vancomycin</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="n"/>
+          <t>piptazo</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>4.5 g q6h</t>
+        </is>
+      </c>
       <c r="C96" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D96" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>15-20 mg/kg q 12 h</t>
-        </is>
-      </c>
-      <c r="G96" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="H96" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="I96" s="2" t="inlineStr">
-        <is>
-          <t>q 12 h</t>
-        </is>
-      </c>
-      <c r="J96" s="2" t="inlineStr">
-        <is>
-          <t>20-25 mg/kg ครั้งเดียว — เฉพาะผู้ป่วยวิกฤตที่สงสัย/ยืนยันติดเชื้อ MRSA รุนแรง; คิดตามน้ำหนักจริง; สูงสุด 3 g; เริ่มขนาดคงระดับในรอบถัดไป</t>
-        </is>
-      </c>
+          <t>4.5 g q 12 h หรือ 2.25 g q 6 h</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="n"/>
+      <c r="H96" s="2" t="n"/>
+      <c r="I96" s="2" t="n"/>
+      <c r="J96" s="2" t="n"/>
       <c r="K96" s="2" t="n"/>
       <c r="L96" s="2" t="inlineStr">
         <is>
           <t>ตรวจสอบ</t>
         </is>
       </c>
-      <c r="N96" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5081,33 +5075,33 @@
       </c>
       <c r="B97" s="2" t="n"/>
       <c r="C97" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D97" s="2" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>50</v>
+        <v>9999</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>10-15 mg/kg q 24 h</t>
+          <t>15-20 mg/kg q 8-12 h</t>
         </is>
       </c>
       <c r="G97" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>q 24 h</t>
+          <t>q 8-12 h</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>20-25 mg/kg ครั้งเดียว — เฉพาะผู้ป่วยวิกฤตที่สงสัย/ยืนยันติดเชื้อ MRSA รุนแรง; คิดตามน้ำหนักจริง; สูงสุด 3 g; เริ่มขนาดคงระดับในรอบถัดไป</t>
+          <t>25-30 mg/kg ครั้งเดียว — เฉพาะผู้ป่วยวิกฤตที่สงสัย/ยืนยันติดเชื้อ MRSA รุนแรง; คิดตามน้ำหนักจริง; สูงสุด 3 g; เริ่มขนาดคงระดับในรอบถัดไป</t>
         </is>
       </c>
       <c r="K97" s="2" t="n"/>
@@ -5116,6 +5110,11 @@
           <t>ตรวจสอบ</t>
         </is>
       </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5125,28 +5124,28 @@
       </c>
       <c r="B98" s="2" t="n"/>
       <c r="C98" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D98" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E98" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>15-20 mg/kg q 12 h</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="E98" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>10-15 mg/kg q 24 h</t>
-        </is>
-      </c>
-      <c r="G98" s="2" t="n">
-        <v>10</v>
-      </c>
       <c r="H98" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>q 24 h</t>
+          <t>q 12 h</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -5160,6 +5159,11 @@
           <t>ตรวจสอบ</t>
         </is>
       </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -5169,17 +5173,17 @@
       </c>
       <c r="B99" s="2" t="n"/>
       <c r="C99" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D99" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>10-15 mg/kg q 48-72 h</t>
+          <t>10-15 mg/kg q 24 h</t>
         </is>
       </c>
       <c r="G99" s="2" t="n">
@@ -5190,7 +5194,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>q 48-72 h</t>
+          <t>q 24 h</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -5208,28 +5212,40 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>amphotericinB</t>
+          <t>vancomycin</t>
         </is>
       </c>
       <c r="B100" s="2" t="n"/>
       <c r="C100" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D100" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>9999</v>
+        <v>30</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาดตาม CrCl (ระวังพิษต่อไต — ดูหมายเหตุ/การติดตาม)</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="n"/>
-      <c r="H100" s="2" t="n"/>
-      <c r="I100" s="2" t="n"/>
-      <c r="J100" s="2" t="n"/>
+          <t>10-15 mg/kg q 24 h</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H100" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>q 24 h</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>20-25 mg/kg ครั้งเดียว — เฉพาะผู้ป่วยวิกฤตที่สงสัย/ยืนยันติดเชื้อ MRSA รุนแรง; คิดตามน้ำหนักจริง; สูงสุด 3 g; เริ่มขนาดคงระดับในรอบถัดไป</t>
+        </is>
+      </c>
       <c r="K100" s="2" t="n"/>
       <c r="L100" s="2" t="inlineStr">
         <is>
@@ -5240,28 +5256,40 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>cloxacillin</t>
+          <t>vancomycin</t>
         </is>
       </c>
       <c r="B101" s="2" t="n"/>
       <c r="C101" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D101" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>9999</v>
+        <v>15</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด</t>
-        </is>
-      </c>
-      <c r="G101" s="2" t="n"/>
-      <c r="H101" s="2" t="n"/>
-      <c r="I101" s="2" t="n"/>
-      <c r="J101" s="2" t="n"/>
+          <t>10-15 mg/kg q 48-72 h</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H101" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>q 48-72 h</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>20-25 mg/kg ครั้งเดียว — เฉพาะผู้ป่วยวิกฤตที่สงสัย/ยืนยันติดเชื้อ MRSA รุนแรง; คิดตามน้ำหนักจริง; สูงสุด 3 g; เริ่มขนาดคงระดับในรอบถัดไป</t>
+        </is>
+      </c>
       <c r="K101" s="2" t="n"/>
       <c r="L101" s="2" t="inlineStr">
         <is>
@@ -5272,7 +5300,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>metronidazole</t>
+          <t>amphotericinB</t>
         </is>
       </c>
       <c r="B102" s="2" t="n"/>
@@ -5287,7 +5315,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>ไม่ต้องปรับขนาด</t>
+          <t>ไม่ต้องปรับขนาดตาม CrCl (ระวังพิษต่อไต — ดูหมายเหตุ/การติดตาม)</t>
         </is>
       </c>
       <c r="G102" s="2" t="n"/>
@@ -5304,7 +5332,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>ceftriaxone</t>
+          <t>cloxacillin</t>
         </is>
       </c>
       <c r="B103" s="2" t="n"/>
@@ -5336,7 +5364,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>clindamycin</t>
+          <t>metronidazole</t>
         </is>
       </c>
       <c r="B104" s="2" t="n"/>
@@ -5368,7 +5396,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>remdesivir</t>
+          <t>ceftriaxone</t>
         </is>
       </c>
       <c r="B105" s="2" t="n"/>
@@ -5392,6 +5420,70 @@
       <c r="J105" s="2" t="n"/>
       <c r="K105" s="2" t="n"/>
       <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>ตรวจสอบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>clindamycin</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="n"/>
+      <c r="C106" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" s="2" t="n">
+        <v>9999</v>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>ไม่ต้องปรับขนาด</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="n"/>
+      <c r="H106" s="2" t="n"/>
+      <c r="I106" s="2" t="n"/>
+      <c r="J106" s="2" t="n"/>
+      <c r="K106" s="2" t="n"/>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>ตรวจสอบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>remdesivir</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="n"/>
+      <c r="C107" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>9999</v>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>ไม่ต้องปรับขนาด</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="n"/>
+      <c r="H107" s="2" t="n"/>
+      <c r="I107" s="2" t="n"/>
+      <c r="J107" s="2" t="n"/>
+      <c r="K107" s="2" t="n"/>
+      <c r="L107" s="2" t="inlineStr">
         <is>
           <t>ตรวจสอบ</t>
         </is>

</xml_diff>

<commit_message>
Amikacin conventional CrCl >=60: show the two valid dose pairs
The helper merged 5 mg/kg q8h and 7.5 mg/kg q12h into "5-7.5 mg/kg ... q 8-12 h",
which reads as up to 7.5 mg/kg q8h (22.5 mg/kg/day). It now shows e.g.
"300 mg q 8 h หรือ 450 mg q 12 h". Rules workbook gains column mgkg_pairs.
Reference table unchanged (no mg calculation; regimens already listed separately).
sw.js CACHE renal-v5.

Fixes #3

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/App/IV-ATB-Renal-App_RULES.xlsx
+++ b/App/IV-ATB-Renal-App_RULES.xlsx
@@ -1408,7 +1408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N107"/>
+  <dimension ref="A1:O107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1494,6 +1494,11 @@
           <t>upper_inclusive</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>mgkg_pairs</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1536,6 +1541,11 @@
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>ตรวจสอบ</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>5:q 8 h|7.5:q 12 h</t>
         </is>
       </c>
     </row>

</xml_diff>